<commit_message>
Rework the МДК.05.03 plan before writing lessons
- rename practices so they no longer repeat lecture titles
- add lectures on database and interface testing
- shorten the defect and documentation practices to keep 96 hours
- move the organization lecture after the new topics and renumber the plan
</commit_message>
<xml_diff>
--- a/courses/3/is-testing/dist/Учебный_план_Тестирование_информационных_систем.xlsx
+++ b/courses/3/is-testing/dist/Учебный_план_Тестирование_информационных_систем.xlsx
@@ -109,7 +109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -307,7 +307,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 1. Тест-план; Классы эквивалентности</t>
+          <t xml:space="preserve">Практика 1. План тестирования учебной системы</t>
         </is>
       </c>
       <c r="D10" s="6">
@@ -397,7 +397,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 2. Граничные значения; Тест-кейсы</t>
+          <t xml:space="preserve">Практика 2. Набор проверок для формы приёмки</t>
         </is>
       </c>
       <c r="D13" s="6">
@@ -487,7 +487,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 3. Чек-лист; Тестирование требований</t>
+          <t xml:space="preserve">Практика 3. Проверка требований к складу</t>
         </is>
       </c>
       <c r="D16" s="6">
@@ -577,7 +577,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 4. Функциональные тесты; Интеграционные тесты</t>
+          <t xml:space="preserve">Практика 4. Сквозные сценарии приёмки и отгрузки</t>
         </is>
       </c>
       <c r="D19" s="6">
@@ -637,7 +637,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 5. Системные тесты</t>
+          <t xml:space="preserve">Практика 5. Проверка системы целиком на стенде</t>
         </is>
       </c>
       <c r="D21" s="6">
@@ -697,7 +697,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 6. Регрессия</t>
+          <t xml:space="preserve">Практика 6. Набор проверок после обновления</t>
         </is>
       </c>
       <c r="D23" s="6">
@@ -787,7 +787,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 7. API-тесты; Postman: коллекция</t>
+          <t xml:space="preserve">Практика 7. Коллекция запросов к API склада</t>
         </is>
       </c>
       <c r="D26" s="6">
@@ -817,7 +817,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 8. Postman: тесты 200/500/JSON</t>
+          <t xml:space="preserve">Практика 8. Проверки ответов API в Postman</t>
         </is>
       </c>
       <c r="D27" s="6">
@@ -877,7 +877,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 9. Автотесты</t>
+          <t xml:space="preserve">Практика 9. Первый набор автотестов на pytest</t>
         </is>
       </c>
       <c r="D29" s="6">
@@ -967,7 +967,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 10. Нагрузка; Безопасность</t>
+          <t xml:space="preserve">Практика 10. Проверка нагрузки и доступа</t>
         </is>
       </c>
       <c r="D32" s="6">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 11. Юзабилити</t>
+          <t xml:space="preserve">Практика 11. Оценка удобства интерфейса склада</t>
         </is>
       </c>
       <c r="D34" s="6">
@@ -1077,7 +1077,7 @@
     <row r="36" ht="60" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">37-38</t>
+          <t xml:space="preserve">37</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
@@ -1087,11 +1087,11 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 12. Баг-репорт; Bug tracking</t>
+          <t xml:space="preserve">Практика 12. Журнал дефектов учебной системы</t>
         </is>
       </c>
       <c r="D36" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
     <row r="37" ht="45" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">39</t>
+          <t xml:space="preserve">38</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
@@ -1137,7 +1137,7 @@
     <row r="38" ht="45" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">40-41</t>
+          <t xml:space="preserve">39</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
@@ -1147,11 +1147,11 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 13. Отчёт; Тестовая документация</t>
+          <t xml:space="preserve">Практика 13. Итоговая документация тестирования</t>
         </is>
       </c>
       <c r="D38" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
     <row r="39" ht="60" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">42</t>
+          <t xml:space="preserve">40</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 21. Организация тестирования</t>
+          <t xml:space="preserve">Лекция 21. Тестирование баз данных</t>
         </is>
       </c>
       <c r="D39" s="6">
@@ -1185,49 +1185,49 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тестирование встраивается в работу команды: роли, уровни, вход и выход из этапов. Разбираются стратегия, оценка трудозатрат и работа с рисками качества.</t>
+          <t xml:space="preserve">Проверка схемы, ограничений, транзакций и самих данных: как найти дубликат, потерянную связь и неверный тип. Вы построите набор запросов, которые проверяют базу склада и объясняют результат.</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">стратегия, роль, оценка, риск, процесс, метрика</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="45" customHeight="1">
+          <t xml:space="preserve">схема, ограничение, дубликат, потерянная связь, транзакция, откат</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="60" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">43-44</t>
+          <t xml:space="preserve">41</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 14. Тестирование БД; Тестирование интерфейса</t>
+          <t xml:space="preserve">Лекция 22. Тестирование интерфейса</t>
         </is>
       </c>
       <c r="D40" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы проверяете сохранение данных в БД и работу интерфейса учебной ИС. Сдаёте SQL-запросы проверки данных и набор тестов интерфейса с результатами.</t>
+          <t xml:space="preserve">Проверка экранов склада: обязательные поля, состояния кнопок, сообщения об ошибках и работа с клавиатуры. Вы составите набор проверок интерфейса и найдёте дефекты, которые не видны в API.</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">целостность данных, SQL-проверка, валидация поля, расхождение, транзакция</t>
+          <t xml:space="preserve">экран, обязательное поле, сообщение об ошибке, состояние элемента, клавиатура, доступность</t>
         </is>
       </c>
     </row>
     <row r="41" ht="45" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">45</t>
+          <t xml:space="preserve">42-43</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -1237,37 +1237,37 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 15. Тестирование интеграций</t>
+          <t xml:space="preserve">Практика 14. Проверка данных и интерфейса</t>
         </is>
       </c>
       <c r="D41" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы проверяете обмен учебной ИС с внешним сервисом и поведение при сбое. Сдаёте набор тестов интеграции и отчёт об обработке ошибок.</t>
+          <t xml:space="preserve">Вы проверяете сохранение данных в БД и работу интерфейса учебной ИС. Сдаёте SQL-запросы проверки данных и набор тестов интерфейса с результатами.</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">внешний сервис, таймаут, повтор, идемпотентность, очередь</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="45" customHeight="1">
+          <t xml:space="preserve">целостность данных, SQL-проверка, валидация поля, расхождение, транзакция</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="60" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">46</t>
+          <t xml:space="preserve">44</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 16. Мини-проект</t>
+          <t xml:space="preserve">Лекция 23. Организация тестирования</t>
         </is>
       </c>
       <c r="D42" s="6">
@@ -1275,112 +1275,172 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вы проводите цикл тестирования небольшой ИС от плана до отчёта. Сдаёте пакет документов и защищаете принятые решения по объёму проверок.</t>
+          <t xml:space="preserve">Тестирование встраивается в работу команды: роли, уровни, вход и выход из этапов. Разбираются стратегия, оценка трудозатрат и работа с рисками качества.</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">цикл тестирования, план, дефект, отчёт, защита</t>
+          <t xml:space="preserve">стратегия, роль, оценка, риск, процесс, метрика</t>
         </is>
       </c>
     </row>
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">45</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 15. Обмен данными между складом и бухгалтерией</t>
+        </is>
+      </c>
+      <c r="D43" s="6">
+        <v>2</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вы проверяете обмен учебной ИС с внешним сервисом и поведение при сбое. Сдаёте набор тестов интеграции и отчёт об обработке ошибок.</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">внешний сервис, таймаут, повтор, идемпотентность, очередь</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="45" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">46</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 16. Мини-проект: тестирование модуля</t>
+        </is>
+      </c>
+      <c r="D44" s="6">
+        <v>2</v>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Вы проводите цикл тестирования небольшой ИС от плана до отчёта. Сдаёте пакет документов и защищаете принятые решения по объёму проверок.</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">цикл тестирования, план, дефект, отчёт, защита</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="45" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">47</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 17. Итоговый отчёт</t>
-        </is>
-      </c>
-      <c r="D43" s="6">
-        <v>2</v>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 17. Сводный отчёт по проекту</t>
+        </is>
+      </c>
+      <c r="D45" s="6">
+        <v>2</v>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Вы сводите результаты проверок в итоговый отчёт с метриками и выводом о готовности. Сдаёте отчёт и презентацию для защиты.</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">метрика, готовность, презентация, вывод, сводка</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="60" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">48</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Практика 18. Защита</t>
-        </is>
-      </c>
-      <c r="D44" s="6">
-        <v>2</v>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика 18. Защита проекта</t>
+        </is>
+      </c>
+      <c r="D46" s="6">
+        <v>2</v>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Вы защищаете результаты тестирования учебной ИС: объём проверок, найденные дефекты и вывод о качестве. Сдаёте доклад и отвечаете на вопросы по решениям.</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">доклад, обоснование, вопросы, качество, вывод</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="7" t="inlineStr">
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Итого</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="D45" s="6">
+      <c r="D47" s="6">
         <v>96</v>
       </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">39 позиций</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">41 позиция</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:F44"/>
+  <autoFilter ref="A5:F46"/>
   <mergeCells count="4">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A47:C47"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>